<commit_message>
fix DepartmentPill styling types
</commit_message>
<xml_diff>
--- a/exam_schedule.xlsx
+++ b/exam_schedule.xlsx
@@ -5,15 +5,15 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="FSC" sheetId="1" state="visible" r:id="rId3"/>
     <sheet name="FSM" sheetId="2" state="visible" r:id="rId4"/>
-    <sheet name="EE" sheetId="3" state="visible" r:id="rId5"/>
+    <sheet name="FSE" sheetId="3" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="false" localSheetId="2" name="_xlnm.Print_Area" vbProcedure="false">EE!$A$1:$L$18</definedName>
+    <definedName function="false" hidden="false" localSheetId="2" name="_xlnm.Print_Area" vbProcedure="false">FSE!$A$1:$L$18</definedName>
     <definedName function="false" hidden="false" localSheetId="1" name="_xlnm.Print_Area" vbProcedure="false">FSM!$A$1:$N$22</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
@@ -616,7 +616,7 @@
   </si>
   <si>
     <t xml:space="preserve">SS2041 Critical Thinking
-BFT-4A,B,C,D
+BS(FT)-4A,B,C,D
 2024</t>
   </si>
   <si>
@@ -696,9 +696,9 @@
   </si>
   <si>
     <t xml:space="preserve">SS2006 Macro Economics
-BAF-4A,B,C
+BS(AF)-4A,B,C
 BBA-4A,B,C
-BSBA-4A,B,C
+BS(BA)-4A,B,C
 2024</t>
   </si>
   <si>
@@ -749,12 +749,12 @@
   </si>
   <si>
     <t xml:space="preserve">BA2006 Fundamentals of Business Analytics
-B(BA)-4A,B,C
+BS(BA)-4A,B,C
 2024</t>
   </si>
   <si>
     <t xml:space="preserve">SS2019 Psychology
-BAF-2A,B
+BS(AF)-2A,B
 2025</t>
   </si>
   <si>
@@ -789,7 +789,7 @@
   <si>
     <t xml:space="preserve">SS2008 Business Communication–I
 BBA-8A
-BSBA-8A
+BS(BA)-8A
 2022</t>
   </si>
   <si>
@@ -799,7 +799,7 @@
   </si>
   <si>
     <t xml:space="preserve">AF2001 Corporate Accounting – I
-B(AF)-4A
+BS(AF)-4A
 2024</t>
   </si>
   <si>
@@ -842,7 +842,7 @@
   </si>
   <si>
     <t xml:space="preserve">MG3033-Principles of Leadership
-BAF-8A
+BS(AF)-8A
 2022</t>
   </si>
   <si>
@@ -852,7 +852,7 @@
   </si>
   <si>
     <t xml:space="preserve">AF2002 Corporate Accounting – II
-B(AF)-4A,B,C
+BS(AF)-4A,B,C
 2024</t>
   </si>
   <si>
@@ -876,7 +876,7 @@
   </si>
   <si>
     <t xml:space="preserve">MG4002 Communication for Managers
-BFT-8A
+BS(FT)-8A
 2022</t>
   </si>
   <si>
@@ -902,7 +902,7 @@
   </si>
   <si>
     <t xml:space="preserve">SS1013 Ideology and Constitution of Pakistan
-BFT-4A,B,C,D
+BS(FT)-4A,B,C,D
 2024</t>
   </si>
   <si>
@@ -935,7 +935,7 @@
   </si>
   <si>
     <t xml:space="preserve">AF4013 Artificial Intelligence in Business Decision
-BFT-8A, 8B
+BS(FT)-8A, 8B
 2022</t>
   </si>
   <si>
@@ -945,7 +945,7 @@
   </si>
   <si>
     <t xml:space="preserve">SS1015 Pakistan Studies
-B(AF)-4A,B,C
+BS(AF)-4A,B,C
 BBA-4A,B,C
 BS(BA)-4A,B,C
 2024</t>
@@ -1003,18 +1003,18 @@
   </si>
   <si>
     <t xml:space="preserve">CS2018 Operating Systems
-BEE-6A,B
+BS(EE)-6A,B
 2023</t>
   </si>
   <si>
     <t xml:space="preserve">EE1005 Digital Logic Design
-BCE-4A
-BEE-4A,B
+BS(CE)-4A
+BS(EE)-4A,B
 2024</t>
   </si>
   <si>
     <t xml:space="preserve">EE3003 Analogue and Digital Communication
-BEE-6A
+BS(EE)-6A
 2023</t>
   </si>
   <si>
@@ -1022,7 +1022,7 @@
   </si>
   <si>
     <t xml:space="preserve">CS2002 Data Structures and Algorithms
-BCE-4A
+BS(CE)-4A
 2024</t>
   </si>
   <si>
@@ -1032,17 +1032,17 @@
   </si>
   <si>
     <t xml:space="preserve">EE4033 Industrial Processes Control 
-BEE-8A
+BS(EE)-8A
 2022</t>
   </si>
   <si>
     <t xml:space="preserve">ME2001 Basic Mechanical Engineering
-BEE-6A
+BS(EE)-6A
 2023</t>
   </si>
   <si>
     <t xml:space="preserve">CS1002 Programming Fundamentals
-BEE-4A
+BS(EE)-4A
 2024</t>
   </si>
   <si>
@@ -1052,7 +1052,7 @@
   </si>
   <si>
     <t xml:space="preserve">EE3031 Digital Signal Processing 
-BEE-6A
+BS(EE)-6A
 2023</t>
   </si>
   <si>
@@ -1063,12 +1063,12 @@
   </si>
   <si>
     <t xml:space="preserve">EE4031 Computer Architecture
-BEE-6A,B
+BS(EE)-6A,B
 2023</t>
   </si>
   <si>
     <t xml:space="preserve">EE2011 Probability and Random Processes
-BEE-4A,B,C
+BS(EE)-4A,B,C
 2024</t>
   </si>
   <si>
@@ -1078,22 +1078,22 @@
   </si>
   <si>
     <t xml:space="preserve">EE3032 Power Electronics
-BEE-6A
+BS(EE)-6A
 2023</t>
   </si>
   <si>
     <t xml:space="preserve">MT2005 Probability and Statistics
-BCE-4A
+BS(CE)-4A
 2024</t>
   </si>
   <si>
     <t xml:space="preserve">IO3031 Introduction to Internet of Things
-BEE-8A
+BS(EE)-8A
 2022</t>
   </si>
   <si>
     <t xml:space="preserve">MG3008 Engineering Economics
-BEE-6A,B
+BS(EE)-6A,B
 2023</t>
   </si>
   <si>
@@ -1104,12 +1104,12 @@
   </si>
   <si>
     <t xml:space="preserve">CS2021 Object Oriented Data Structures
-BEE-4A
+BS(EE)-4A
 2024</t>
   </si>
   <si>
     <t xml:space="preserve">SS2010 Communication Skills
-BEE-6A,B
+BS(EE)-6A,B
 2023</t>
   </si>
   <si>
@@ -1119,19 +1119,19 @@
   </si>
   <si>
     <t xml:space="preserve">SS2011  Technical Communication Skills
-BCE-4A
-BEE-4A,B
+BS(CE)-4A
+BS(EE)-4A,B
 2024</t>
   </si>
   <si>
     <t xml:space="preserve">MG4011 Entrepreneurship
-BEE-8A
-BEE-8B
+BS(EE)-8A
+BS(EE)-8B
 2022</t>
   </si>
   <si>
     <t xml:space="preserve">EE3004 Feedback Control System
-BEE-6A,B
+BS(EE)-6A,B
 2023</t>
   </si>
   <si>
@@ -1141,43 +1141,43 @@
   </si>
   <si>
     <t xml:space="preserve">EE3034 VLSI
-BEE-8A
+BS(EE)-8A
 2022</t>
   </si>
   <si>
     <t xml:space="preserve">EE2004 Electrical Network Analysis
-BEE-4A,B
+BS(EE)-4A,B
 2024</t>
   </si>
   <si>
     <t xml:space="preserve">EE2015 Electro-Mechanical Systems
-BEE-4A,B
+BS(EE)-4A,B
 2024</t>
   </si>
   <si>
     <t xml:space="preserve">EE4043 Network Programming
-BEE-8A
+BS(EE)-8A
 2022</t>
   </si>
   <si>
     <t xml:space="preserve">EE2010 Electro-Mechanical Systems
-BEE-6A,B
+BS(EE)-6A,B
 2023</t>
   </si>
   <si>
     <t xml:space="preserve">EE2008 Signals and Systems 
-BCE-4A
-BEE-4A,B
+BS(CE)-4A
+BS(EE)-4A,B
 2024</t>
   </si>
   <si>
     <t xml:space="preserve">MT1009 Linear Algebra and Diff. Equations
-BEE-4A
+BS(EE)-4A
 2024</t>
   </si>
   <si>
     <t xml:space="preserve">NS1007 Applied Physics
-BEE-2A
+BS(EE)-2A
 2025</t>
   </si>
 </sst>
@@ -1191,7 +1191,7 @@
     <numFmt numFmtId="166" formatCode="h:mm\ AM/PM"/>
     <numFmt numFmtId="167" formatCode="[$-F800]dddd&quot;, &quot;mmmm\ dd&quot;, &quot;yyyy"/>
   </numFmts>
-  <fonts count="37">
+  <fonts count="35">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -1332,11 +1332,6 @@
       <charset val="1"/>
     </font>
     <font>
-      <sz val="14"/>
-      <name val="Arial"/>
-      <family val="2"/>
-    </font>
-    <font>
       <sz val="18"/>
       <name val="Times New Roman"/>
       <family val="1"/>
@@ -1390,12 +1385,6 @@
       <name val="Times New Roman"/>
       <family val="1"/>
       <charset val="1"/>
-    </font>
-    <font>
-      <sz val="16"/>
-      <color theme="1"/>
-      <name val="Times New Roman"/>
-      <family val="1"/>
     </font>
     <font>
       <sz val="16"/>
@@ -1719,892 +1708,884 @@
       <protection locked="true" hidden="false"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="222">
+  <cellXfs count="220">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="8" fillId="2" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="9" fillId="2" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="9" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="11" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="167" fontId="12" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="8" fillId="2" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="9" fillId="2" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="9" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="12" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="90" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="13" fillId="3" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="13" fillId="4" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="13" fillId="3" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="13" fillId="4" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="13" fillId="5" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="13" fillId="6" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="13" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="13" fillId="5" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="13" fillId="6" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="13" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="13" fillId="7" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="14" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="13" fillId="7" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="14" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="14" fillId="4" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="14" fillId="4" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="14" fillId="0" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="13" fillId="8" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="13" fillId="7" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="13" fillId="9" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="13" fillId="10" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="13" fillId="11" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="14" fillId="0" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="13" fillId="0" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="15" fillId="12" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="13" fillId="0" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="14" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="13" fillId="0" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="14" fillId="0" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="167" fontId="12" fillId="0" borderId="8" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="14" fillId="0" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="13" fillId="8" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="13" fillId="7" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="13" fillId="9" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="13" fillId="10" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="13" fillId="11" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="14" fillId="0" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="13" fillId="0" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="15" fillId="12" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="13" fillId="0" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="14" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="13" fillId="0" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="14" fillId="0" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="12" fillId="0" borderId="8" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="center" textRotation="90" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="167" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="center" textRotation="90" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="167" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="90" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="12" fillId="0" borderId="9" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="167" fontId="12" fillId="0" borderId="9" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="center" textRotation="90" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="14" fillId="0" borderId="9" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="13" fillId="0" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="14" fillId="0" borderId="9" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="13" fillId="0" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="16" fillId="0" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="16" fillId="0" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="45" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="13" fillId="5" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="13" fillId="5" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="14" fillId="0" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="14" fillId="0" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="13" fillId="6" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="15" fillId="13" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="13" fillId="0" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="13" fillId="6" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="15" fillId="13" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="13" fillId="0" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="14" fillId="0" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="14" fillId="0" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="13" fillId="3" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="14" fillId="0" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="13" fillId="0" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="13" fillId="3" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="14" fillId="0" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="13" fillId="0" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="14" fillId="0" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="14" fillId="0" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="13" fillId="4" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="13" fillId="4" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="13" fillId="5" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="14" fillId="4" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="13" fillId="5" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="14" fillId="4" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="15" fillId="13" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="13" fillId="4" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="15" fillId="13" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="13" fillId="4" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="14" fillId="4" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="14" fillId="4" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="13" fillId="10" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="13" fillId="4" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="13" fillId="10" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="13" fillId="4" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="14" fillId="4" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="14" fillId="4" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="12" fillId="0" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="167" fontId="12" fillId="0" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="90" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="13" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="13" fillId="0" borderId="10" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="13" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="13" fillId="0" borderId="10" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="21" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="21" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="167" fontId="21" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="21" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="21" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="21" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="90" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="14" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="17" fillId="0" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="10" fillId="15" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="17" fillId="0" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="10" fillId="16" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="11" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="10" fillId="15" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="5" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="17" fillId="17" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="14" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="17" fillId="0" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="15" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="17" fillId="0" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="16" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="11" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="15" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="5" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="17" fillId="17" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="17" fillId="0" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="10" fillId="18" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="8" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="8" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="10" fillId="19" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="10" fillId="20" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="17" fillId="0" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="18" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="8" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="8" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="19" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="20" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="17" fillId="21" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="17" fillId="0" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="12" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="7" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="167" fontId="21" fillId="0" borderId="8" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="17" fillId="21" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="17" fillId="0" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="12" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="7" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="21" fillId="0" borderId="8" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="center" textRotation="90" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="167" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="center" textRotation="90" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="21" fillId="0" borderId="9" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="167" fontId="21" fillId="0" borderId="9" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="center" textRotation="90" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="16" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="16" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="45" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="10" fillId="18" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="10" fillId="16" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="10" fillId="14" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="10" fillId="17" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="6" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="167" fontId="21" fillId="0" borderId="13" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="18" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="16" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="14" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="17" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="6" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="21" fillId="0" borderId="13" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="center" textRotation="90" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="21" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="167" fontId="21" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="center" textRotation="90" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="21" fillId="0" borderId="14" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="167" fontId="21" fillId="0" borderId="14" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="center" textRotation="90" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="21" fillId="0" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="167" fontId="21" fillId="0" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="90" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="19" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="11" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="22" fillId="18" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="19" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="11" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="6" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="9" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="167" fontId="21" fillId="0" borderId="11" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="6" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="9" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="21" fillId="0" borderId="11" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="center" textRotation="90" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="21" fillId="0" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="167" fontId="21" fillId="0" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="center" textRotation="90" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="21" fillId="0" borderId="15" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="167" fontId="21" fillId="0" borderId="15" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="center" textRotation="90" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="15" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="15" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="4" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="4" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="22" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="22" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="7" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="26" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="27" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="27" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="28" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="29" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="30" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="30" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="31" fillId="3" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="32" fillId="0" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="33" fillId="7" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="34" fillId="0" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="35" fillId="23" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="34" fillId="0" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="35" fillId="24" borderId="13" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="35" fillId="0" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="32" fillId="11" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="35" fillId="0" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="35" fillId="23" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="32" fillId="3" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="32" fillId="0" borderId="15" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="34" fillId="0" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="34" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="35" fillId="0" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="32" fillId="0" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="35" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="32" fillId="10" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="32" fillId="0" borderId="9" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="35" fillId="0" borderId="9" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="32" fillId="0" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="35" fillId="24" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="32" fillId="0" borderId="10" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="35" fillId="0" borderId="10" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="34" fillId="0" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="35" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="34" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="35" fillId="0" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="32" fillId="0" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="35" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="167" fontId="12" fillId="0" borderId="12" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="7" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="26" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="26" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="27" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="28" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="29" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="29" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="30" fillId="3" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="30" fillId="0" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="31" fillId="7" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="32" fillId="0" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="33" fillId="23" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="32" fillId="0" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="33" fillId="24" borderId="13" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="33" fillId="0" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="30" fillId="11" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="33" fillId="0" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="33" fillId="23" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="30" fillId="3" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="30" fillId="0" borderId="15" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="32" fillId="0" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="32" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="33" fillId="0" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="30" fillId="0" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="33" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="30" fillId="10" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="30" fillId="0" borderId="9" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="33" fillId="0" borderId="9" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="30" fillId="0" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="33" fillId="24" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="30" fillId="0" borderId="10" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="33" fillId="0" borderId="10" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="32" fillId="0" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="33" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="32" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="33" fillId="0" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="30" fillId="0" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="33" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="12" fillId="0" borderId="12" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="center" textRotation="90" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="167" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="center" textRotation="90" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="12" fillId="0" borderId="10" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="167" fontId="12" fillId="0" borderId="10" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="center" textRotation="90" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="32" fillId="3" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="32" fillId="0" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="35" fillId="7" borderId="15" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="32" fillId="7" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="35" fillId="0" borderId="11" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="32" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="35" fillId="0" borderId="8" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="35" fillId="13" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="17" fillId="0" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="35" fillId="0" borderId="8" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="167" fontId="12" fillId="0" borderId="13" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="30" fillId="0" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="33" fillId="7" borderId="15" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="30" fillId="7" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="33" fillId="0" borderId="11" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="30" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="33" fillId="0" borderId="8" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="33" fillId="13" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="17" fillId="0" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="33" fillId="0" borderId="8" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="12" fillId="0" borderId="13" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="center" textRotation="90" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="12" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="167" fontId="12" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="center" textRotation="90" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="12" fillId="0" borderId="14" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="167" fontId="12" fillId="0" borderId="14" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="center" textRotation="90" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="35" fillId="7" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="35" fillId="0" borderId="11" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="35" fillId="12" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="32" fillId="10" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="35" fillId="0" borderId="12" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="32" fillId="0" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="32" fillId="12" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="17" fillId="0" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="17" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="17" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="16" fillId="0" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="36" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="36" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="33" fillId="7" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="33" fillId="0" borderId="11" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="33" fillId="12" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="30" fillId="10" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="33" fillId="0" borderId="12" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="30" fillId="0" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="30" fillId="12" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="17" fillId="0" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="17" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="17" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="16" fillId="0" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="34" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="34" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -5455,7 +5436,7 @@
     </row>
     <row r="19" customFormat="false" ht="105" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="128"/>
-      <c r="B19" s="131" t="s">
+      <c r="B19" s="94" t="s">
         <v>153</v>
       </c>
       <c r="C19" s="92"/>
@@ -5480,12 +5461,12 @@
       <c r="N19" s="119"/>
       <c r="P19" s="123"/>
     </row>
-    <row r="20" s="133" customFormat="true" ht="104.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="20" s="132" customFormat="true" ht="104.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="128"/>
       <c r="B20" s="85" t="s">
         <v>158</v>
       </c>
-      <c r="C20" s="132"/>
+      <c r="C20" s="131"/>
       <c r="D20" s="81" t="s">
         <v>159</v>
       </c>
@@ -5503,52 +5484,52 @@
       </c>
       <c r="M20" s="98"/>
       <c r="N20" s="100"/>
-      <c r="P20" s="134"/>
-    </row>
-    <row r="21" s="133" customFormat="true" ht="87" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="P20" s="133"/>
+    </row>
+    <row r="21" s="132" customFormat="true" ht="87" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="128"/>
-      <c r="C21" s="132"/>
+      <c r="C21" s="131"/>
       <c r="D21" s="81"/>
       <c r="E21" s="118"/>
       <c r="F21" s="18"/>
       <c r="G21" s="118"/>
       <c r="I21" s="95"/>
-      <c r="J21" s="135"/>
+      <c r="J21" s="134"/>
       <c r="K21" s="118"/>
       <c r="M21" s="98"/>
       <c r="N21" s="100"/>
-      <c r="P21" s="134"/>
-    </row>
-    <row r="22" s="133" customFormat="true" ht="87" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="P21" s="133"/>
+    </row>
+    <row r="22" s="132" customFormat="true" ht="87" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="128"/>
-      <c r="C22" s="132"/>
+      <c r="C22" s="131"/>
       <c r="E22" s="118"/>
       <c r="F22" s="18"/>
       <c r="G22" s="118"/>
       <c r="I22" s="95"/>
-      <c r="J22" s="135"/>
+      <c r="J22" s="134"/>
       <c r="K22" s="118"/>
       <c r="M22" s="98"/>
       <c r="N22" s="100"/>
-      <c r="P22" s="134"/>
+      <c r="P22" s="133"/>
     </row>
     <row r="23" customFormat="false" ht="11.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="136"/>
-      <c r="B23" s="137"/>
-      <c r="C23" s="137"/>
-      <c r="D23" s="137"/>
-      <c r="E23" s="137"/>
-      <c r="F23" s="137"/>
-      <c r="G23" s="137"/>
-      <c r="H23" s="137"/>
-      <c r="I23" s="137"/>
-      <c r="J23" s="137"/>
-      <c r="K23" s="137"/>
-      <c r="L23" s="137"/>
-      <c r="M23" s="137"/>
-      <c r="N23" s="138"/>
+      <c r="A23" s="135"/>
+      <c r="B23" s="136"/>
+      <c r="C23" s="136"/>
+      <c r="D23" s="136"/>
+      <c r="E23" s="136"/>
+      <c r="F23" s="136"/>
+      <c r="G23" s="136"/>
+      <c r="H23" s="136"/>
+      <c r="I23" s="136"/>
+      <c r="J23" s="136"/>
+      <c r="K23" s="136"/>
+      <c r="L23" s="136"/>
+      <c r="M23" s="136"/>
+      <c r="N23" s="137"/>
       <c r="O23" s="90"/>
-      <c r="P23" s="139"/>
+      <c r="P23" s="138"/>
     </row>
     <row r="24" customFormat="false" ht="115.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="80" t="n">
@@ -5569,7 +5550,7 @@
       <c r="H24" s="88" t="s">
         <v>165</v>
       </c>
-      <c r="I24" s="140"/>
+      <c r="I24" s="139"/>
       <c r="J24" s="81" t="s">
         <v>166</v>
       </c>
@@ -5589,7 +5570,7 @@
       <c r="B25" s="120" t="s">
         <v>169</v>
       </c>
-      <c r="C25" s="141"/>
+      <c r="C25" s="140"/>
       <c r="D25" s="119"/>
       <c r="E25" s="124"/>
       <c r="F25" s="88" t="s">
@@ -5618,7 +5599,7 @@
       <c r="B26" s="85" t="s">
         <v>175</v>
       </c>
-      <c r="C26" s="141"/>
+      <c r="C26" s="140"/>
       <c r="D26" s="100"/>
       <c r="E26" s="124"/>
       <c r="F26" s="88"/>
@@ -5636,19 +5617,19 @@
       </c>
       <c r="P26" s="101"/>
     </row>
-    <row r="27" s="133" customFormat="true" ht="92.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="27" s="132" customFormat="true" ht="92.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="80"/>
       <c r="B27" s="85" t="s">
         <v>178</v>
       </c>
-      <c r="C27" s="141"/>
+      <c r="C27" s="140"/>
       <c r="D27" s="100"/>
       <c r="E27" s="124"/>
-      <c r="F27" s="142"/>
+      <c r="F27" s="141"/>
       <c r="G27" s="124"/>
-      <c r="H27" s="143"/>
+      <c r="H27" s="142"/>
       <c r="I27" s="124"/>
-      <c r="J27" s="144" t="s">
+      <c r="J27" s="143" t="s">
         <v>179</v>
       </c>
       <c r="K27" s="124"/>
@@ -5657,74 +5638,74 @@
       </c>
       <c r="M27" s="124"/>
       <c r="N27" s="101"/>
-      <c r="P27" s="134"/>
-    </row>
-    <row r="28" s="133" customFormat="true" ht="99" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="P27" s="133"/>
+    </row>
+    <row r="28" s="132" customFormat="true" ht="99" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="80"/>
       <c r="B28" s="85" t="s">
         <v>181</v>
       </c>
-      <c r="C28" s="141"/>
+      <c r="C28" s="140"/>
       <c r="D28" s="108"/>
       <c r="E28" s="124"/>
       <c r="F28" s="110"/>
       <c r="G28" s="124"/>
-      <c r="H28" s="145"/>
+      <c r="H28" s="144"/>
       <c r="I28" s="124"/>
       <c r="J28" s="103"/>
       <c r="K28" s="124"/>
-      <c r="L28" s="146"/>
+      <c r="L28" s="145"/>
       <c r="M28" s="124"/>
-      <c r="N28" s="147"/>
-      <c r="O28" s="146"/>
-      <c r="P28" s="147"/>
+      <c r="N28" s="146"/>
+      <c r="O28" s="145"/>
+      <c r="P28" s="146"/>
     </row>
     <row r="29" s="26" customFormat="true" ht="56.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A29" s="148" t="s">
+      <c r="A29" s="147" t="s">
         <v>102</v>
       </c>
-      <c r="B29" s="148"/>
-      <c r="C29" s="148"/>
-      <c r="D29" s="148"/>
-      <c r="E29" s="148"/>
-      <c r="F29" s="148"/>
-      <c r="G29" s="148"/>
-      <c r="H29" s="148"/>
-      <c r="I29" s="148"/>
-      <c r="J29" s="148"/>
-      <c r="K29" s="148"/>
-      <c r="L29" s="148"/>
-      <c r="M29" s="148"/>
-      <c r="N29" s="148"/>
+      <c r="B29" s="147"/>
+      <c r="C29" s="147"/>
+      <c r="D29" s="147"/>
+      <c r="E29" s="147"/>
+      <c r="F29" s="147"/>
+      <c r="G29" s="147"/>
+      <c r="H29" s="147"/>
+      <c r="I29" s="147"/>
+      <c r="J29" s="147"/>
+      <c r="K29" s="147"/>
+      <c r="L29" s="147"/>
+      <c r="M29" s="147"/>
+      <c r="N29" s="147"/>
     </row>
     <row r="30" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A30" s="149"/>
-      <c r="B30" s="149"/>
-      <c r="C30" s="149"/>
-      <c r="D30" s="149"/>
-      <c r="E30" s="149"/>
-      <c r="F30" s="149"/>
-      <c r="G30" s="149"/>
-      <c r="H30" s="149"/>
-      <c r="I30" s="149"/>
-      <c r="J30" s="149"/>
-      <c r="K30" s="149"/>
-      <c r="L30" s="149"/>
-      <c r="M30" s="149"/>
-      <c r="N30" s="149"/>
+      <c r="A30" s="148"/>
+      <c r="B30" s="148"/>
+      <c r="C30" s="148"/>
+      <c r="D30" s="148"/>
+      <c r="E30" s="148"/>
+      <c r="F30" s="148"/>
+      <c r="G30" s="148"/>
+      <c r="H30" s="148"/>
+      <c r="I30" s="148"/>
+      <c r="J30" s="148"/>
+      <c r="K30" s="148"/>
+      <c r="L30" s="148"/>
+      <c r="M30" s="148"/>
+      <c r="N30" s="148"/>
     </row>
     <row r="31" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A31" s="150"/>
-      <c r="B31" s="151"/>
-      <c r="C31" s="149"/>
-      <c r="D31" s="149"/>
-      <c r="E31" s="149"/>
-      <c r="F31" s="149"/>
-      <c r="G31" s="149"/>
-      <c r="H31" s="149"/>
-      <c r="I31" s="149"/>
-      <c r="J31" s="149"/>
-      <c r="K31" s="149"/>
+      <c r="A31" s="149"/>
+      <c r="B31" s="150"/>
+      <c r="C31" s="148"/>
+      <c r="D31" s="148"/>
+      <c r="E31" s="148"/>
+      <c r="F31" s="148"/>
+      <c r="G31" s="148"/>
+      <c r="H31" s="148"/>
+      <c r="I31" s="148"/>
+      <c r="J31" s="148"/>
+      <c r="K31" s="148"/>
       <c r="L31" s="71"/>
       <c r="M31" s="71"/>
       <c r="N31" s="71" t="s">
@@ -5732,34 +5713,34 @@
       </c>
     </row>
     <row r="32" s="75" customFormat="true" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A32" s="152"/>
-      <c r="B32" s="151"/>
-      <c r="C32" s="153"/>
-      <c r="D32" s="153"/>
-      <c r="E32" s="153"/>
-      <c r="G32" s="154"/>
-      <c r="H32" s="155" t="s">
+      <c r="A32" s="151"/>
+      <c r="B32" s="150"/>
+      <c r="C32" s="152"/>
+      <c r="D32" s="152"/>
+      <c r="E32" s="152"/>
+      <c r="G32" s="153"/>
+      <c r="H32" s="154" t="s">
         <v>182</v>
       </c>
-      <c r="I32" s="155"/>
-      <c r="J32" s="155"/>
-      <c r="K32" s="155"/>
-      <c r="L32" s="156"/>
+      <c r="I32" s="154"/>
+      <c r="J32" s="154"/>
+      <c r="K32" s="154"/>
+      <c r="L32" s="155"/>
       <c r="M32" s="71"/>
-      <c r="N32" s="156" t="s">
+      <c r="N32" s="155" t="s">
         <v>104</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="70.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="G33" s="154"/>
+      <c r="G33" s="153"/>
       <c r="H33" s="2" t="s">
         <v>182</v>
       </c>
-      <c r="I33" s="155"/>
-      <c r="K33" s="155"/>
-      <c r="L33" s="155"/>
-      <c r="M33" s="155"/>
-      <c r="N33" s="155"/>
+      <c r="I33" s="154"/>
+      <c r="K33" s="154"/>
+      <c r="L33" s="154"/>
+      <c r="M33" s="154"/>
+      <c r="N33" s="154"/>
     </row>
     <row r="35" s="75" customFormat="true" ht="18.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D35" s="73"/>
@@ -5841,56 +5822,56 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="37.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="157" t="s">
+      <c r="A1" s="156" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="157"/>
-      <c r="C1" s="157"/>
-      <c r="D1" s="157"/>
-      <c r="E1" s="157"/>
-      <c r="F1" s="157"/>
-      <c r="G1" s="157"/>
-      <c r="H1" s="157"/>
-      <c r="I1" s="157"/>
-      <c r="J1" s="157"/>
-      <c r="K1" s="157"/>
-      <c r="L1" s="157"/>
+      <c r="B1" s="156"/>
+      <c r="C1" s="156"/>
+      <c r="D1" s="156"/>
+      <c r="E1" s="156"/>
+      <c r="F1" s="156"/>
+      <c r="G1" s="156"/>
+      <c r="H1" s="156"/>
+      <c r="I1" s="156"/>
+      <c r="J1" s="156"/>
+      <c r="K1" s="156"/>
+      <c r="L1" s="156"/>
     </row>
     <row r="2" customFormat="false" ht="37.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="158" t="s">
+      <c r="A2" s="157" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="158"/>
-      <c r="C2" s="158"/>
-      <c r="D2" s="158"/>
-      <c r="E2" s="158"/>
-      <c r="F2" s="158"/>
-      <c r="G2" s="158"/>
-      <c r="H2" s="158"/>
-      <c r="I2" s="158"/>
-      <c r="J2" s="158"/>
-      <c r="K2" s="158"/>
-      <c r="L2" s="158"/>
+      <c r="B2" s="157"/>
+      <c r="C2" s="157"/>
+      <c r="D2" s="157"/>
+      <c r="E2" s="157"/>
+      <c r="F2" s="157"/>
+      <c r="G2" s="157"/>
+      <c r="H2" s="157"/>
+      <c r="I2" s="157"/>
+      <c r="J2" s="157"/>
+      <c r="K2" s="157"/>
+      <c r="L2" s="157"/>
     </row>
     <row r="3" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="159" t="s">
+      <c r="A3" s="158" t="s">
         <v>183</v>
       </c>
-      <c r="B3" s="159"/>
-      <c r="C3" s="159"/>
-      <c r="D3" s="159"/>
-      <c r="E3" s="159"/>
-      <c r="F3" s="159"/>
-      <c r="G3" s="159"/>
-      <c r="H3" s="159"/>
-      <c r="I3" s="159"/>
-      <c r="J3" s="159"/>
-      <c r="K3" s="160"/>
+      <c r="B3" s="158"/>
+      <c r="C3" s="158"/>
+      <c r="D3" s="158"/>
+      <c r="E3" s="158"/>
+      <c r="F3" s="158"/>
+      <c r="G3" s="158"/>
+      <c r="H3" s="158"/>
+      <c r="I3" s="158"/>
+      <c r="J3" s="158"/>
+      <c r="K3" s="159"/>
       <c r="L3" s="7" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="4" s="161" customFormat="true" ht="73.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="4" s="160" customFormat="true" ht="73.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="8" t="s">
         <v>4</v>
       </c>
@@ -5922,401 +5903,401 @@
       <c r="A5" s="15" t="n">
         <v>46121</v>
       </c>
-      <c r="B5" s="162" t="s">
+      <c r="B5" s="161" t="s">
         <v>184</v>
       </c>
-      <c r="C5" s="163"/>
-      <c r="D5" s="164" t="s">
+      <c r="C5" s="162"/>
+      <c r="D5" s="163" t="s">
         <v>185</v>
       </c>
-      <c r="E5" s="165"/>
-      <c r="F5" s="166" t="s">
+      <c r="E5" s="164"/>
+      <c r="F5" s="165" t="s">
         <v>186</v>
       </c>
-      <c r="G5" s="167"/>
-      <c r="H5" s="168" t="s">
+      <c r="G5" s="166"/>
+      <c r="H5" s="167" t="s">
         <v>187</v>
       </c>
-      <c r="I5" s="169"/>
-      <c r="J5" s="170" t="s">
+      <c r="I5" s="168"/>
+      <c r="J5" s="169" t="s">
         <v>188</v>
       </c>
-      <c r="K5" s="171"/>
-      <c r="L5" s="172" t="s">
+      <c r="K5" s="170"/>
+      <c r="L5" s="171" t="s">
         <v>189</v>
       </c>
     </row>
     <row r="6" s="73" customFormat="true" ht="113.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="15"/>
-      <c r="B6" s="173" t="s">
+      <c r="B6" s="172" t="s">
         <v>190</v>
       </c>
-      <c r="C6" s="174"/>
-      <c r="D6" s="164"/>
-      <c r="E6" s="175"/>
-      <c r="F6" s="166"/>
-      <c r="G6" s="176"/>
-      <c r="H6" s="169"/>
-      <c r="I6" s="177"/>
-      <c r="J6" s="178"/>
-      <c r="K6" s="179"/>
-      <c r="L6" s="180" t="s">
+      <c r="C6" s="173"/>
+      <c r="D6" s="163"/>
+      <c r="E6" s="174"/>
+      <c r="F6" s="165"/>
+      <c r="G6" s="175"/>
+      <c r="H6" s="168"/>
+      <c r="I6" s="176"/>
+      <c r="J6" s="177"/>
+      <c r="K6" s="178"/>
+      <c r="L6" s="179" t="s">
         <v>191</v>
       </c>
     </row>
     <row r="7" s="73" customFormat="true" ht="113.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="15"/>
-      <c r="B7" s="173"/>
-      <c r="C7" s="181"/>
-      <c r="D7" s="182"/>
-      <c r="E7" s="175"/>
-      <c r="F7" s="166"/>
-      <c r="G7" s="176"/>
-      <c r="H7" s="177"/>
-      <c r="I7" s="177"/>
-      <c r="J7" s="183"/>
-      <c r="K7" s="179"/>
-      <c r="L7" s="184" t="s">
+      <c r="B7" s="172"/>
+      <c r="C7" s="180"/>
+      <c r="D7" s="181"/>
+      <c r="E7" s="174"/>
+      <c r="F7" s="165"/>
+      <c r="G7" s="175"/>
+      <c r="H7" s="176"/>
+      <c r="I7" s="176"/>
+      <c r="J7" s="182"/>
+      <c r="K7" s="178"/>
+      <c r="L7" s="183" t="s">
         <v>192</v>
       </c>
     </row>
     <row r="8" s="73" customFormat="true" ht="113.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="15"/>
-      <c r="B8" s="170" t="s">
+      <c r="B8" s="169" t="s">
         <v>193</v>
       </c>
-      <c r="C8" s="185"/>
-      <c r="D8" s="186"/>
-      <c r="E8" s="187"/>
-      <c r="F8" s="188"/>
-      <c r="G8" s="189"/>
-      <c r="H8" s="190"/>
-      <c r="I8" s="190"/>
-      <c r="J8" s="191"/>
-      <c r="K8" s="192"/>
-      <c r="L8" s="173"/>
+      <c r="C8" s="184"/>
+      <c r="D8" s="185"/>
+      <c r="E8" s="186"/>
+      <c r="F8" s="187"/>
+      <c r="G8" s="188"/>
+      <c r="H8" s="189"/>
+      <c r="I8" s="189"/>
+      <c r="J8" s="190"/>
+      <c r="K8" s="191"/>
+      <c r="L8" s="172"/>
     </row>
     <row r="9" s="73" customFormat="true" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="193"/>
-      <c r="B9" s="194"/>
-      <c r="C9" s="194"/>
-      <c r="D9" s="194"/>
-      <c r="E9" s="194"/>
-      <c r="F9" s="194"/>
-      <c r="G9" s="194"/>
-      <c r="H9" s="194"/>
-      <c r="I9" s="194"/>
-      <c r="J9" s="194"/>
-      <c r="K9" s="194"/>
-      <c r="L9" s="195"/>
+      <c r="A9" s="192"/>
+      <c r="B9" s="193"/>
+      <c r="C9" s="193"/>
+      <c r="D9" s="193"/>
+      <c r="E9" s="193"/>
+      <c r="F9" s="193"/>
+      <c r="G9" s="193"/>
+      <c r="H9" s="193"/>
+      <c r="I9" s="193"/>
+      <c r="J9" s="193"/>
+      <c r="K9" s="193"/>
+      <c r="L9" s="194"/>
     </row>
     <row r="10" s="73" customFormat="true" ht="104.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="15" t="n">
         <v>46122</v>
       </c>
-      <c r="B10" s="196" t="s">
+      <c r="B10" s="161" t="s">
         <v>194</v>
       </c>
-      <c r="C10" s="197"/>
-      <c r="D10" s="198" t="s">
+      <c r="C10" s="195"/>
+      <c r="D10" s="196" t="s">
         <v>195</v>
       </c>
-      <c r="E10" s="165"/>
-      <c r="F10" s="173" t="s">
+      <c r="E10" s="164"/>
+      <c r="F10" s="172" t="s">
         <v>196</v>
       </c>
-      <c r="G10" s="165"/>
+      <c r="G10" s="164"/>
       <c r="H10" s="114" t="s">
         <v>33</v>
       </c>
-      <c r="I10" s="169"/>
-      <c r="J10" s="199" t="s">
+      <c r="I10" s="168"/>
+      <c r="J10" s="197" t="s">
         <v>197</v>
       </c>
-      <c r="K10" s="200"/>
-      <c r="L10" s="172" t="s">
+      <c r="K10" s="198"/>
+      <c r="L10" s="171" t="s">
         <v>198</v>
       </c>
     </row>
     <row r="11" s="73" customFormat="true" ht="104.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="15"/>
-      <c r="B11" s="196" t="s">
+      <c r="B11" s="161" t="s">
         <v>199</v>
       </c>
-      <c r="C11" s="201"/>
-      <c r="D11" s="198"/>
-      <c r="E11" s="175"/>
-      <c r="F11" s="173"/>
-      <c r="G11" s="175"/>
+      <c r="C11" s="199"/>
+      <c r="D11" s="196"/>
+      <c r="E11" s="174"/>
+      <c r="F11" s="172"/>
+      <c r="G11" s="174"/>
       <c r="H11" s="114"/>
-      <c r="I11" s="177"/>
-      <c r="J11" s="199" t="s">
+      <c r="I11" s="176"/>
+      <c r="J11" s="197" t="s">
         <v>200</v>
       </c>
-      <c r="K11" s="202"/>
-      <c r="L11" s="166" t="s">
+      <c r="K11" s="200"/>
+      <c r="L11" s="165" t="s">
         <v>201</v>
       </c>
     </row>
     <row r="12" s="73" customFormat="true" ht="104.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="15"/>
-      <c r="B12" s="180" t="s">
+      <c r="B12" s="179" t="s">
         <v>202</v>
       </c>
-      <c r="C12" s="201"/>
-      <c r="D12" s="169"/>
-      <c r="E12" s="175"/>
-      <c r="F12" s="178"/>
-      <c r="G12" s="175"/>
+      <c r="C12" s="199"/>
+      <c r="D12" s="168"/>
+      <c r="E12" s="174"/>
+      <c r="F12" s="177"/>
+      <c r="G12" s="174"/>
       <c r="H12" s="114"/>
-      <c r="I12" s="177"/>
-      <c r="J12" s="178"/>
-      <c r="K12" s="202"/>
-      <c r="L12" s="203"/>
+      <c r="I12" s="176"/>
+      <c r="J12" s="177"/>
+      <c r="K12" s="200"/>
+      <c r="L12" s="201"/>
     </row>
     <row r="13" s="73" customFormat="true" ht="104.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="15"/>
-      <c r="B13" s="204"/>
-      <c r="C13" s="201"/>
-      <c r="D13" s="190"/>
-      <c r="E13" s="175"/>
-      <c r="F13" s="191"/>
-      <c r="G13" s="175"/>
+      <c r="B13" s="202"/>
+      <c r="C13" s="199"/>
+      <c r="D13" s="189"/>
+      <c r="E13" s="174"/>
+      <c r="F13" s="190"/>
+      <c r="G13" s="174"/>
       <c r="H13" s="114"/>
-      <c r="I13" s="177"/>
-      <c r="J13" s="191"/>
-      <c r="K13" s="205"/>
-      <c r="L13" s="203"/>
+      <c r="I13" s="176"/>
+      <c r="J13" s="190"/>
+      <c r="K13" s="203"/>
+      <c r="L13" s="201"/>
     </row>
     <row r="14" s="73" customFormat="true" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="206"/>
-      <c r="B14" s="207"/>
-      <c r="C14" s="207"/>
-      <c r="D14" s="207"/>
-      <c r="E14" s="207"/>
-      <c r="F14" s="207"/>
-      <c r="G14" s="207"/>
-      <c r="H14" s="207"/>
-      <c r="I14" s="207"/>
-      <c r="J14" s="207"/>
-      <c r="K14" s="207"/>
-      <c r="L14" s="208"/>
+      <c r="A14" s="204"/>
+      <c r="B14" s="205"/>
+      <c r="C14" s="205"/>
+      <c r="D14" s="205"/>
+      <c r="E14" s="205"/>
+      <c r="F14" s="205"/>
+      <c r="G14" s="205"/>
+      <c r="H14" s="205"/>
+      <c r="I14" s="205"/>
+      <c r="J14" s="205"/>
+      <c r="K14" s="205"/>
+      <c r="L14" s="206"/>
     </row>
     <row r="15" s="73" customFormat="true" ht="133.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="15" t="n">
         <v>46123</v>
       </c>
-      <c r="B15" s="209" t="s">
+      <c r="B15" s="207" t="s">
         <v>203</v>
       </c>
-      <c r="C15" s="210"/>
-      <c r="D15" s="173" t="s">
+      <c r="C15" s="208"/>
+      <c r="D15" s="172" t="s">
         <v>204</v>
       </c>
-      <c r="E15" s="165"/>
-      <c r="F15" s="211" t="s">
+      <c r="E15" s="164"/>
+      <c r="F15" s="209" t="s">
         <v>205</v>
       </c>
-      <c r="G15" s="167"/>
-      <c r="H15" s="199" t="s">
+      <c r="G15" s="166"/>
+      <c r="H15" s="197" t="s">
         <v>206</v>
       </c>
-      <c r="I15" s="169"/>
-      <c r="J15" s="170" t="s">
+      <c r="I15" s="168"/>
+      <c r="J15" s="169" t="s">
         <v>207</v>
       </c>
-      <c r="K15" s="169"/>
-      <c r="L15" s="172" t="s">
+      <c r="K15" s="168"/>
+      <c r="L15" s="171" t="s">
         <v>208</v>
       </c>
     </row>
     <row r="16" s="73" customFormat="true" ht="110.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="15"/>
-      <c r="B16" s="209"/>
-      <c r="C16" s="205"/>
-      <c r="D16" s="173"/>
-      <c r="E16" s="175"/>
-      <c r="F16" s="211"/>
-      <c r="G16" s="176"/>
-      <c r="H16" s="199"/>
-      <c r="I16" s="177"/>
-      <c r="K16" s="177"/>
-      <c r="L16" s="212" t="s">
+      <c r="B16" s="207"/>
+      <c r="C16" s="203"/>
+      <c r="D16" s="172"/>
+      <c r="E16" s="174"/>
+      <c r="F16" s="209"/>
+      <c r="G16" s="175"/>
+      <c r="H16" s="197"/>
+      <c r="I16" s="176"/>
+      <c r="K16" s="176"/>
+      <c r="L16" s="210" t="s">
         <v>209</v>
       </c>
     </row>
     <row r="17" s="73" customFormat="true" ht="110.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="15"/>
-      <c r="B17" s="169"/>
-      <c r="C17" s="205"/>
-      <c r="D17" s="178"/>
-      <c r="E17" s="175"/>
-      <c r="F17" s="169"/>
-      <c r="G17" s="176"/>
-      <c r="H17" s="178"/>
-      <c r="I17" s="177"/>
-      <c r="K17" s="177"/>
-      <c r="L17" s="203"/>
+      <c r="B17" s="168"/>
+      <c r="C17" s="203"/>
+      <c r="D17" s="177"/>
+      <c r="E17" s="174"/>
+      <c r="F17" s="168"/>
+      <c r="G17" s="175"/>
+      <c r="H17" s="177"/>
+      <c r="I17" s="176"/>
+      <c r="K17" s="176"/>
+      <c r="L17" s="201"/>
     </row>
     <row r="18" s="73" customFormat="true" ht="110.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="15"/>
-      <c r="B18" s="190"/>
-      <c r="C18" s="213"/>
-      <c r="D18" s="191"/>
-      <c r="E18" s="175"/>
-      <c r="F18" s="190"/>
-      <c r="G18" s="176"/>
-      <c r="H18" s="191"/>
-      <c r="I18" s="177"/>
-      <c r="K18" s="177"/>
-      <c r="L18" s="203"/>
+      <c r="B18" s="189"/>
+      <c r="C18" s="211"/>
+      <c r="D18" s="190"/>
+      <c r="E18" s="174"/>
+      <c r="F18" s="189"/>
+      <c r="G18" s="175"/>
+      <c r="H18" s="190"/>
+      <c r="I18" s="176"/>
+      <c r="K18" s="176"/>
+      <c r="L18" s="201"/>
     </row>
     <row r="19" s="73" customFormat="true" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="206"/>
-      <c r="B19" s="207"/>
-      <c r="C19" s="207"/>
-      <c r="D19" s="207"/>
-      <c r="E19" s="207"/>
-      <c r="F19" s="207"/>
-      <c r="G19" s="207"/>
-      <c r="H19" s="207"/>
-      <c r="I19" s="207"/>
-      <c r="J19" s="207"/>
-      <c r="K19" s="207"/>
-      <c r="L19" s="208"/>
+      <c r="A19" s="204"/>
+      <c r="B19" s="205"/>
+      <c r="C19" s="205"/>
+      <c r="D19" s="205"/>
+      <c r="E19" s="205"/>
+      <c r="F19" s="205"/>
+      <c r="G19" s="205"/>
+      <c r="H19" s="205"/>
+      <c r="I19" s="205"/>
+      <c r="J19" s="205"/>
+      <c r="K19" s="205"/>
+      <c r="L19" s="206"/>
     </row>
     <row r="20" s="73" customFormat="true" ht="87.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="15" t="n">
         <v>46125</v>
       </c>
-      <c r="B20" s="209" t="s">
+      <c r="B20" s="207" t="s">
         <v>210</v>
       </c>
-      <c r="C20" s="163"/>
-      <c r="D20" s="173" t="s">
+      <c r="C20" s="162"/>
+      <c r="D20" s="172" t="s">
         <v>211</v>
       </c>
-      <c r="E20" s="165"/>
-      <c r="F20" s="180" t="s">
+      <c r="E20" s="164"/>
+      <c r="F20" s="179" t="s">
         <v>212</v>
       </c>
-      <c r="G20" s="167"/>
-      <c r="H20" s="211" t="s">
+      <c r="G20" s="166"/>
+      <c r="H20" s="209" t="s">
         <v>213</v>
       </c>
-      <c r="I20" s="169"/>
-      <c r="J20" s="178"/>
-      <c r="K20" s="169"/>
-      <c r="L20" s="166" t="s">
+      <c r="I20" s="168"/>
+      <c r="J20" s="177"/>
+      <c r="K20" s="168"/>
+      <c r="L20" s="165" t="s">
         <v>214</v>
       </c>
     </row>
     <row r="21" s="73" customFormat="true" ht="86.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="15"/>
-      <c r="B21" s="209"/>
-      <c r="C21" s="214"/>
-      <c r="D21" s="173"/>
-      <c r="E21" s="175"/>
-      <c r="F21" s="180" t="s">
+      <c r="B21" s="207"/>
+      <c r="C21" s="212"/>
+      <c r="D21" s="172"/>
+      <c r="E21" s="174"/>
+      <c r="F21" s="179" t="s">
         <v>215</v>
       </c>
-      <c r="G21" s="176"/>
-      <c r="H21" s="211"/>
-      <c r="I21" s="177"/>
-      <c r="J21" s="183"/>
-      <c r="K21" s="177"/>
-      <c r="L21" s="164" t="s">
+      <c r="G21" s="175"/>
+      <c r="H21" s="209"/>
+      <c r="I21" s="176"/>
+      <c r="J21" s="182"/>
+      <c r="K21" s="176"/>
+      <c r="L21" s="163" t="s">
         <v>216</v>
       </c>
     </row>
     <row r="22" s="73" customFormat="true" ht="91.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="15"/>
-      <c r="B22" s="166" t="s">
+      <c r="B22" s="165" t="s">
         <v>217</v>
       </c>
-      <c r="C22" s="163"/>
-      <c r="D22" s="215" t="s">
+      <c r="C22" s="162"/>
+      <c r="D22" s="213" t="s">
         <v>218</v>
       </c>
-      <c r="E22" s="175"/>
-      <c r="F22" s="216"/>
-      <c r="G22" s="176"/>
+      <c r="E22" s="174"/>
+      <c r="F22" s="214"/>
+      <c r="G22" s="175"/>
       <c r="H22" s="82"/>
-      <c r="I22" s="177"/>
-      <c r="J22" s="183"/>
-      <c r="K22" s="177"/>
-      <c r="L22" s="170" t="s">
+      <c r="I22" s="176"/>
+      <c r="J22" s="182"/>
+      <c r="K22" s="176"/>
+      <c r="L22" s="169" t="s">
         <v>219</v>
       </c>
     </row>
     <row r="23" s="73" customFormat="true" ht="91.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="15"/>
-      <c r="B23" s="217"/>
-      <c r="D23" s="190"/>
-      <c r="E23" s="187"/>
-      <c r="F23" s="204"/>
-      <c r="G23" s="189"/>
-      <c r="H23" s="204"/>
-      <c r="I23" s="190"/>
-      <c r="J23" s="218"/>
-      <c r="K23" s="190"/>
-      <c r="L23" s="191"/>
+      <c r="B23" s="215"/>
+      <c r="D23" s="189"/>
+      <c r="E23" s="186"/>
+      <c r="F23" s="202"/>
+      <c r="G23" s="188"/>
+      <c r="H23" s="202"/>
+      <c r="I23" s="189"/>
+      <c r="J23" s="216"/>
+      <c r="K23" s="189"/>
+      <c r="L23" s="190"/>
     </row>
     <row r="24" customFormat="false" ht="69.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="219" t="s">
+      <c r="A24" s="217" t="s">
         <v>102</v>
       </c>
-      <c r="B24" s="219"/>
-      <c r="C24" s="219"/>
-      <c r="D24" s="219"/>
-      <c r="E24" s="219"/>
-      <c r="F24" s="219"/>
-      <c r="G24" s="219"/>
-      <c r="H24" s="219"/>
-      <c r="I24" s="219"/>
-      <c r="J24" s="219"/>
-      <c r="K24" s="219"/>
-      <c r="L24" s="219"/>
+      <c r="B24" s="217"/>
+      <c r="C24" s="217"/>
+      <c r="D24" s="217"/>
+      <c r="E24" s="217"/>
+      <c r="F24" s="217"/>
+      <c r="G24" s="217"/>
+      <c r="H24" s="217"/>
+      <c r="I24" s="217"/>
+      <c r="J24" s="217"/>
+      <c r="K24" s="217"/>
+      <c r="L24" s="217"/>
     </row>
     <row r="25" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="220"/>
-      <c r="B25" s="220"/>
-      <c r="C25" s="220"/>
-      <c r="D25" s="220"/>
-      <c r="E25" s="220"/>
-      <c r="G25" s="220"/>
-      <c r="H25" s="220"/>
-      <c r="I25" s="220"/>
-      <c r="J25" s="220"/>
-      <c r="K25" s="220"/>
-      <c r="L25" s="220"/>
+      <c r="A25" s="218"/>
+      <c r="B25" s="218"/>
+      <c r="C25" s="218"/>
+      <c r="D25" s="218"/>
+      <c r="E25" s="218"/>
+      <c r="G25" s="218"/>
+      <c r="H25" s="218"/>
+      <c r="I25" s="218"/>
+      <c r="J25" s="218"/>
+      <c r="K25" s="218"/>
+      <c r="L25" s="218"/>
     </row>
     <row r="26" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A26" s="220"/>
-      <c r="E26" s="220"/>
-      <c r="F26" s="220"/>
-      <c r="G26" s="220"/>
-      <c r="H26" s="220"/>
-      <c r="I26" s="220"/>
-      <c r="J26" s="220"/>
-      <c r="K26" s="220"/>
-      <c r="L26" s="220"/>
+      <c r="A26" s="218"/>
+      <c r="E26" s="218"/>
+      <c r="F26" s="218"/>
+      <c r="G26" s="218"/>
+      <c r="H26" s="218"/>
+      <c r="I26" s="218"/>
+      <c r="J26" s="218"/>
+      <c r="K26" s="218"/>
+      <c r="L26" s="218"/>
     </row>
     <row r="27" customFormat="false" ht="33" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A27" s="221"/>
-      <c r="E27" s="221"/>
-      <c r="G27" s="221"/>
-      <c r="I27" s="221"/>
+      <c r="A27" s="219"/>
+      <c r="E27" s="219"/>
+      <c r="G27" s="219"/>
+      <c r="I27" s="219"/>
       <c r="L27" s="71" t="s">
         <v>103</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="33" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A28" s="221"/>
+      <c r="A28" s="219"/>
       <c r="D28" s="26"/>
-      <c r="E28" s="221"/>
-      <c r="G28" s="221"/>
-      <c r="I28" s="221"/>
+      <c r="E28" s="219"/>
+      <c r="G28" s="219"/>
+      <c r="I28" s="219"/>
       <c r="L28" s="71" t="s">
         <v>104</v>
       </c>

</xml_diff>

<commit_message>
update exam schedule data in exam_schedule.xlsx
</commit_message>
<xml_diff>
--- a/exam_schedule.xlsx
+++ b/exam_schedule.xlsx
@@ -1135,9 +1135,10 @@
 2023</t>
   </si>
   <si>
-    <t xml:space="preserve">MT1006 Differential Equations  BS(CE) -AB
+    <t xml:space="preserve">MT1006 Differential Equations  
+BS(CE) -AB
 BS(EE) -ABC, BS(CS) R
- 2025</t>
+2025</t>
   </si>
   <si>
     <t xml:space="preserve">EE3034 VLSI

</xml_diff>